<commit_message>
Refactor player movement and visibility logic for enhanced gameplay experience
- Updated the `Player` class to improve movement responsiveness and interaction with the game environment.
- Enhanced visibility calculations to better integrate with the player's effective sight range, ensuring a more immersive fog-of-war experience.
- Streamlined player state updates during movement to optimize performance and reduce latency in gameplay interactions.
</commit_message>
<xml_diff>
--- a/monster_types.xlsx
+++ b/monster_types.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\info\Documents\Projects\dungeon-console\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28B4C1BA-0507-476A-80BC-9BE07C3679FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6756B322-48A6-4494-8AEE-2AF6D26F96C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Monsters" sheetId="1" r:id="rId1"/>
@@ -329,7 +329,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="124">
   <si>
     <t>type_id</t>
   </si>
@@ -599,6 +599,108 @@
   </si>
   <si>
     <t>/static/monsters/portraits/ogre.png</t>
+  </si>
+  <si>
+    <t>caveBat</t>
+  </si>
+  <si>
+    <t>Cave Bat</t>
+  </si>
+  <si>
+    <t>cave bat</t>
+  </si>
+  <si>
+    <t>giantRat</t>
+  </si>
+  <si>
+    <t>Giant Rat</t>
+  </si>
+  <si>
+    <t>giant rat</t>
+  </si>
+  <si>
+    <t>/static/monsters/sprites/caveBat.png</t>
+  </si>
+  <si>
+    <t>/static/monsters/portraits/caveBat.png</t>
+  </si>
+  <si>
+    <t>/static/monsters/portraits/giantRat.png</t>
+  </si>
+  <si>
+    <t>/static/monsters/sprites/giantRat.png</t>
+  </si>
+  <si>
+    <t>goblin</t>
+  </si>
+  <si>
+    <t>Goblin</t>
+  </si>
+  <si>
+    <t>/static/monsters/sprites/goblin.png</t>
+  </si>
+  <si>
+    <t>/static/monsters/portraits/goblin.png</t>
+  </si>
+  <si>
+    <t>poisonMushroom</t>
+  </si>
+  <si>
+    <t>Poison Mushroom</t>
+  </si>
+  <si>
+    <t>/static/monsters/sprites/poisonMushroom.png</t>
+  </si>
+  <si>
+    <t>/static/monsters/portraits/poisonMushroom.png</t>
+  </si>
+  <si>
+    <t>giantSnake</t>
+  </si>
+  <si>
+    <t>Giant Snake</t>
+  </si>
+  <si>
+    <t>/static/monsters/sprites/giantSnake.png</t>
+  </si>
+  <si>
+    <t>/static/monsters/portraits/giantSnake.png</t>
+  </si>
+  <si>
+    <t>imp</t>
+  </si>
+  <si>
+    <t>Imp</t>
+  </si>
+  <si>
+    <t>/static/monsters/sprites/imp.png</t>
+  </si>
+  <si>
+    <t>/static/monsters/portraits/imp.png</t>
+  </si>
+  <si>
+    <t>giantBeetle</t>
+  </si>
+  <si>
+    <t>Giant Beetle</t>
+  </si>
+  <si>
+    <t>/static/monsters/sprites/giantBeetle.png</t>
+  </si>
+  <si>
+    <t>/static/monsters/portraits/giantBeetle.png</t>
+  </si>
+  <si>
+    <t>mummy</t>
+  </si>
+  <si>
+    <t>Mummy</t>
+  </si>
+  <si>
+    <t>/static/monsters/sprites/mummy.png</t>
+  </si>
+  <si>
+    <t>/static/monsters/portraits/mummy.png</t>
   </si>
 </sst>
 </file>
@@ -1132,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="O2" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P2" s="2">
         <v>20</v>
@@ -1195,7 +1297,7 @@
         <v>10</v>
       </c>
       <c r="O3" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P3" s="2">
         <v>20</v>
@@ -1207,7 +1309,7 @@
       <c r="S3" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="T3" s="3">
+      <c r="T3" s="2">
         <v>0.5</v>
       </c>
       <c r="U3" s="2" t="s">
@@ -1270,7 +1372,7 @@
       <c r="S4" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="T4" s="3">
+      <c r="T4" s="2">
         <v>0.5</v>
       </c>
       <c r="U4" s="2" t="s">
@@ -1333,7 +1435,7 @@
       <c r="S5" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="T5" s="3">
+      <c r="T5" s="2">
         <v>0.5</v>
       </c>
       <c r="U5" s="2" t="s">
@@ -1396,196 +1498,516 @@
       <c r="S6" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="T6" s="3">
+      <c r="T6" s="2">
         <v>0.5</v>
       </c>
       <c r="U6" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
-      <c r="O7" s="3"/>
-      <c r="P7" s="3"/>
+    <row r="7" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="D7" s="3">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2">
+        <v>8</v>
+      </c>
+      <c r="F7" s="2">
+        <v>3</v>
+      </c>
+      <c r="G7" s="2">
+        <v>3</v>
+      </c>
+      <c r="H7" s="2">
+        <v>2</v>
+      </c>
+      <c r="I7" s="2">
+        <v>4</v>
+      </c>
+      <c r="J7" s="2">
+        <v>4</v>
+      </c>
+      <c r="K7" s="2">
+        <v>6</v>
+      </c>
+      <c r="L7" s="2">
+        <v>10</v>
+      </c>
+      <c r="M7" s="2">
+        <v>5</v>
+      </c>
+      <c r="N7" s="2">
+        <v>10</v>
+      </c>
+      <c r="O7" s="2">
+        <v>1</v>
+      </c>
+      <c r="P7" s="2">
+        <v>20</v>
+      </c>
       <c r="Q7" s="3"/>
-      <c r="R7" s="3"/>
-      <c r="S7" s="3"/>
-      <c r="T7" s="3"/>
-      <c r="U7" s="3"/>
-    </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
-      <c r="M8" s="3"/>
-      <c r="N8" s="3"/>
-      <c r="O8" s="3"/>
-      <c r="P8" s="3"/>
+      <c r="R7" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="S7" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="T7" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="U7" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="D8" s="3">
+        <v>1</v>
+      </c>
+      <c r="E8" s="2">
+        <v>8</v>
+      </c>
+      <c r="F8" s="2">
+        <v>3</v>
+      </c>
+      <c r="G8" s="2">
+        <v>3</v>
+      </c>
+      <c r="H8" s="2">
+        <v>2</v>
+      </c>
+      <c r="I8" s="2">
+        <v>4</v>
+      </c>
+      <c r="J8" s="2">
+        <v>4</v>
+      </c>
+      <c r="K8" s="2">
+        <v>6</v>
+      </c>
+      <c r="L8" s="2">
+        <v>10</v>
+      </c>
+      <c r="M8" s="2">
+        <v>5</v>
+      </c>
+      <c r="N8" s="2">
+        <v>10</v>
+      </c>
+      <c r="O8" s="2">
+        <v>10</v>
+      </c>
+      <c r="P8" s="2">
+        <v>20</v>
+      </c>
       <c r="Q8" s="3"/>
-      <c r="R8" s="3"/>
-      <c r="S8" s="3"/>
-      <c r="T8" s="3"/>
-      <c r="U8" s="3"/>
-    </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
-      <c r="O9" s="3"/>
-      <c r="P9" s="3"/>
+      <c r="R8" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="S8" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="T8" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="U8" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="D9" s="3">
+        <v>1</v>
+      </c>
+      <c r="E9" s="2">
+        <v>8</v>
+      </c>
+      <c r="F9" s="2">
+        <v>3</v>
+      </c>
+      <c r="G9" s="2">
+        <v>3</v>
+      </c>
+      <c r="H9" s="2">
+        <v>2</v>
+      </c>
+      <c r="I9" s="2">
+        <v>4</v>
+      </c>
+      <c r="J9" s="2">
+        <v>4</v>
+      </c>
+      <c r="K9" s="2">
+        <v>6</v>
+      </c>
+      <c r="L9" s="2">
+        <v>10</v>
+      </c>
+      <c r="M9" s="2">
+        <v>5</v>
+      </c>
+      <c r="N9" s="2">
+        <v>10</v>
+      </c>
+      <c r="O9" s="2">
+        <v>5</v>
+      </c>
+      <c r="P9" s="2">
+        <v>20</v>
+      </c>
       <c r="Q9" s="3"/>
-      <c r="R9" s="3"/>
-      <c r="S9" s="3"/>
-      <c r="T9" s="3"/>
-      <c r="U9" s="3"/>
-    </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
-      <c r="M10" s="3"/>
-      <c r="N10" s="3"/>
-      <c r="O10" s="3"/>
-      <c r="P10" s="3"/>
+      <c r="R9" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="S9" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="T9" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="U9" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="D10" s="3">
+        <v>1</v>
+      </c>
+      <c r="E10" s="2">
+        <v>8</v>
+      </c>
+      <c r="F10" s="2">
+        <v>3</v>
+      </c>
+      <c r="G10" s="2">
+        <v>3</v>
+      </c>
+      <c r="H10" s="2">
+        <v>2</v>
+      </c>
+      <c r="I10" s="2">
+        <v>4</v>
+      </c>
+      <c r="J10" s="2">
+        <v>4</v>
+      </c>
+      <c r="K10" s="2">
+        <v>6</v>
+      </c>
+      <c r="L10" s="2">
+        <v>10</v>
+      </c>
+      <c r="M10" s="2">
+        <v>5</v>
+      </c>
+      <c r="N10" s="2">
+        <v>10</v>
+      </c>
+      <c r="O10" s="2">
+        <v>4</v>
+      </c>
+      <c r="P10" s="2">
+        <v>20</v>
+      </c>
       <c r="Q10" s="3"/>
-      <c r="R10" s="3"/>
-      <c r="S10" s="3"/>
-      <c r="T10" s="3"/>
-      <c r="U10" s="3"/>
-    </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
-      <c r="L11" s="3"/>
-      <c r="M11" s="3"/>
-      <c r="N11" s="3"/>
-      <c r="O11" s="3"/>
-      <c r="P11" s="3"/>
+      <c r="R10" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="S10" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="T10" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="U10" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="D11" s="3">
+        <v>1</v>
+      </c>
+      <c r="E11" s="2">
+        <v>8</v>
+      </c>
+      <c r="F11" s="2">
+        <v>3</v>
+      </c>
+      <c r="G11" s="2">
+        <v>3</v>
+      </c>
+      <c r="H11" s="2">
+        <v>2</v>
+      </c>
+      <c r="I11" s="2">
+        <v>4</v>
+      </c>
+      <c r="J11" s="2">
+        <v>4</v>
+      </c>
+      <c r="K11" s="2">
+        <v>6</v>
+      </c>
+      <c r="L11" s="2">
+        <v>10</v>
+      </c>
+      <c r="M11" s="2">
+        <v>5</v>
+      </c>
+      <c r="N11" s="2">
+        <v>10</v>
+      </c>
+      <c r="O11" s="2">
+        <v>10</v>
+      </c>
+      <c r="P11" s="2">
+        <v>20</v>
+      </c>
       <c r="Q11" s="3"/>
-      <c r="R11" s="3"/>
-      <c r="S11" s="3"/>
-      <c r="T11" s="3"/>
-      <c r="U11" s="3"/>
-    </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-      <c r="L12" s="3"/>
-      <c r="M12" s="3"/>
-      <c r="N12" s="3"/>
-      <c r="O12" s="3"/>
-      <c r="P12" s="3"/>
+      <c r="R11" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="S11" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="T11" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="U11" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="D12" s="3">
+        <v>1</v>
+      </c>
+      <c r="E12" s="2">
+        <v>8</v>
+      </c>
+      <c r="F12" s="2">
+        <v>3</v>
+      </c>
+      <c r="G12" s="2">
+        <v>3</v>
+      </c>
+      <c r="H12" s="2">
+        <v>2</v>
+      </c>
+      <c r="I12" s="2">
+        <v>4</v>
+      </c>
+      <c r="J12" s="2">
+        <v>4</v>
+      </c>
+      <c r="K12" s="2">
+        <v>6</v>
+      </c>
+      <c r="L12" s="2">
+        <v>10</v>
+      </c>
+      <c r="M12" s="2">
+        <v>5</v>
+      </c>
+      <c r="N12" s="2">
+        <v>10</v>
+      </c>
+      <c r="O12" s="2">
+        <v>1</v>
+      </c>
+      <c r="P12" s="2">
+        <v>20</v>
+      </c>
       <c r="Q12" s="3"/>
-      <c r="R12" s="3"/>
-      <c r="S12" s="3"/>
-      <c r="T12" s="3"/>
-      <c r="U12" s="3"/>
-    </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
-      <c r="M13" s="3"/>
-      <c r="N13" s="3"/>
-      <c r="O13" s="3"/>
-      <c r="P13" s="3"/>
+      <c r="R12" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="S12" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="T12" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="U12" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="D13" s="3">
+        <v>1</v>
+      </c>
+      <c r="E13" s="2">
+        <v>8</v>
+      </c>
+      <c r="F13" s="2">
+        <v>3</v>
+      </c>
+      <c r="G13" s="2">
+        <v>3</v>
+      </c>
+      <c r="H13" s="2">
+        <v>2</v>
+      </c>
+      <c r="I13" s="2">
+        <v>4</v>
+      </c>
+      <c r="J13" s="2">
+        <v>4</v>
+      </c>
+      <c r="K13" s="2">
+        <v>6</v>
+      </c>
+      <c r="L13" s="2">
+        <v>10</v>
+      </c>
+      <c r="M13" s="2">
+        <v>5</v>
+      </c>
+      <c r="N13" s="2">
+        <v>10</v>
+      </c>
+      <c r="O13" s="2">
+        <v>10</v>
+      </c>
+      <c r="P13" s="2">
+        <v>20</v>
+      </c>
       <c r="Q13" s="3"/>
-      <c r="R13" s="3"/>
-      <c r="S13" s="3"/>
-      <c r="T13" s="3"/>
-      <c r="U13" s="3"/>
-    </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
-      <c r="M14" s="3"/>
-      <c r="N14" s="3"/>
-      <c r="O14" s="3"/>
-      <c r="P14" s="3"/>
+      <c r="R13" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="S13" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="T13" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="U13" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="D14" s="3">
+        <v>1</v>
+      </c>
+      <c r="E14" s="2">
+        <v>8</v>
+      </c>
+      <c r="F14" s="2">
+        <v>3</v>
+      </c>
+      <c r="G14" s="2">
+        <v>3</v>
+      </c>
+      <c r="H14" s="2">
+        <v>2</v>
+      </c>
+      <c r="I14" s="2">
+        <v>4</v>
+      </c>
+      <c r="J14" s="2">
+        <v>4</v>
+      </c>
+      <c r="K14" s="2">
+        <v>6</v>
+      </c>
+      <c r="L14" s="2">
+        <v>10</v>
+      </c>
+      <c r="M14" s="2">
+        <v>5</v>
+      </c>
+      <c r="N14" s="2">
+        <v>10</v>
+      </c>
+      <c r="O14" s="2">
+        <v>10</v>
+      </c>
+      <c r="P14" s="2">
+        <v>20</v>
+      </c>
       <c r="Q14" s="3"/>
-      <c r="R14" s="3"/>
-      <c r="S14" s="3"/>
-      <c r="T14" s="3"/>
-      <c r="U14" s="3"/>
+      <c r="R14" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="S14" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="T14" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="U14" s="2" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>

</xml_diff>

<commit_message>
Enhance terrain features and improve map generation logic
- Introduced new terrain types: mountains and walls, enriching the visual diversity of the game map.
- Updated map generation to utilize mountains as borders, enhancing gameplay dynamics and aesthetics.
- Refined visibility logic to accommodate new terrain types, ensuring accurate navigation and interaction.
- Enhanced rendering logic to support new terrain graphics, including mountain and wall sprites.
- Expanded test coverage for terrain interactions and player movement dynamics related to the updated features.
</commit_message>
<xml_diff>
--- a/monster_types.xlsx
+++ b/monster_types.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\info\Documents\Projects\dungeon-console\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6756B322-48A6-4494-8AEE-2AF6D26F96C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{744EB8AD-677D-4548-AC40-CEB8688507D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34200" yWindow="2655" windowWidth="21600" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Monsters" sheetId="1" r:id="rId1"/>
@@ -1562,7 +1562,7 @@
         <v>97</v>
       </c>
       <c r="T7" s="2">
-        <v>0.5</v>
+        <v>100</v>
       </c>
       <c r="U7" s="2" t="s">
         <v>26</v>

</xml_diff>

<commit_message>
Refactor attack damage logic and enhance gameplay dynamics
- Implemented new attack damage calculations to improve combat interactions.
- Updated player and enemy classes to utilize the new damage logic effectively.
- Enhanced test coverage for combat scenarios to ensure accurate damage reporting and interactions.
</commit_message>
<xml_diff>
--- a/monster_types.xlsx
+++ b/monster_types.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\info\Documents\Projects\dungeon-console\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{744EB8AD-677D-4548-AC40-CEB8688507D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{656E5DAD-82F4-4AEB-BB43-73C9FA36DCD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34200" yWindow="2655" windowWidth="21600" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Monsters" sheetId="1" r:id="rId1"/>
@@ -1204,7 +1204,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="2">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F2" s="2">
         <v>3</v>
@@ -1247,7 +1247,7 @@
         <v>25</v>
       </c>
       <c r="T2" s="2">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="U2" s="2" t="s">
         <v>26</v>
@@ -1267,7 +1267,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="2">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F3" s="2">
         <v>3</v>
@@ -1310,7 +1310,7 @@
         <v>75</v>
       </c>
       <c r="T3" s="2">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="U3" s="2" t="s">
         <v>26</v>
@@ -1348,7 +1348,7 @@
         <v>4</v>
       </c>
       <c r="K4" s="2">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="L4" s="2">
         <v>10</v>
@@ -1373,7 +1373,7 @@
         <v>78</v>
       </c>
       <c r="T4" s="2">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="U4" s="2" t="s">
         <v>26</v>
@@ -1393,7 +1393,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="2">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F5" s="2">
         <v>3</v>
@@ -1411,7 +1411,7 @@
         <v>4</v>
       </c>
       <c r="K5" s="2">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="L5" s="2">
         <v>10</v>
@@ -1436,7 +1436,7 @@
         <v>87</v>
       </c>
       <c r="T5" s="2">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="U5" s="2" t="s">
         <v>26</v>
@@ -1456,7 +1456,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="2">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="F6" s="2">
         <v>3</v>
@@ -1474,7 +1474,7 @@
         <v>4</v>
       </c>
       <c r="K6" s="2">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="L6" s="2">
         <v>10</v>
@@ -1499,7 +1499,7 @@
         <v>89</v>
       </c>
       <c r="T6" s="2">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="U6" s="2" t="s">
         <v>26</v>
@@ -1519,7 +1519,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="2">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F7" s="2">
         <v>3</v>
@@ -1537,7 +1537,7 @@
         <v>4</v>
       </c>
       <c r="K7" s="2">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="L7" s="2">
         <v>10</v>
@@ -1562,7 +1562,7 @@
         <v>97</v>
       </c>
       <c r="T7" s="2">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="U7" s="2" t="s">
         <v>26</v>
@@ -1582,7 +1582,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F8" s="2">
         <v>3</v>
@@ -1600,7 +1600,7 @@
         <v>4</v>
       </c>
       <c r="K8" s="2">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="L8" s="2">
         <v>10</v>
@@ -1625,7 +1625,7 @@
         <v>98</v>
       </c>
       <c r="T8" s="2">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="U8" s="2" t="s">
         <v>26</v>
@@ -1645,7 +1645,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F9" s="2">
         <v>3</v>
@@ -1663,7 +1663,7 @@
         <v>4</v>
       </c>
       <c r="K9" s="2">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="L9" s="2">
         <v>10</v>
@@ -1688,7 +1688,7 @@
         <v>103</v>
       </c>
       <c r="T9" s="2">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="U9" s="2" t="s">
         <v>26</v>
@@ -1708,7 +1708,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="2">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F10" s="2">
         <v>3</v>
@@ -1726,7 +1726,7 @@
         <v>4</v>
       </c>
       <c r="K10" s="2">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="L10" s="2">
         <v>10</v>
@@ -1751,7 +1751,7 @@
         <v>107</v>
       </c>
       <c r="T10" s="2">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="U10" s="2" t="s">
         <v>26</v>
@@ -1771,7 +1771,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F11" s="2">
         <v>3</v>
@@ -1789,7 +1789,7 @@
         <v>4</v>
       </c>
       <c r="K11" s="2">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="L11" s="2">
         <v>10</v>
@@ -1814,7 +1814,7 @@
         <v>111</v>
       </c>
       <c r="T11" s="2">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="U11" s="2" t="s">
         <v>26</v>
@@ -1852,7 +1852,7 @@
         <v>4</v>
       </c>
       <c r="K12" s="2">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="L12" s="2">
         <v>10</v>
@@ -1877,7 +1877,7 @@
         <v>115</v>
       </c>
       <c r="T12" s="2">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="U12" s="2" t="s">
         <v>26</v>
@@ -1897,7 +1897,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F13" s="2">
         <v>3</v>
@@ -1915,7 +1915,7 @@
         <v>4</v>
       </c>
       <c r="K13" s="2">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="L13" s="2">
         <v>10</v>
@@ -1940,7 +1940,7 @@
         <v>119</v>
       </c>
       <c r="T13" s="2">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="U13" s="2" t="s">
         <v>26</v>
@@ -1960,7 +1960,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F14" s="2">
         <v>3</v>
@@ -1978,7 +1978,7 @@
         <v>4</v>
       </c>
       <c r="K14" s="2">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="L14" s="2">
         <v>10</v>
@@ -2003,7 +2003,7 @@
         <v>123</v>
       </c>
       <c r="T14" s="2">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="U14" s="2" t="s">
         <v>26</v>

</xml_diff>

<commit_message>
Refactor monster attributes and enhance combat interactions
- Introduced an `armour` attribute to the `MonsterTypeDef` class, ensuring a minimum value of 1 for validation.
- Updated the monster sheet to display the new `armour` attribute and adjusted related documentation.
- Modified the `Monster` class to incorporate the `armour` attribute from the type definition.
- Enhanced unit tests to validate the functionality and parsing of the `armour` attribute in various scenarios.
</commit_message>
<xml_diff>
--- a/monster_types.xlsx
+++ b/monster_types.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\info\Documents\Projects\dungeon-console\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{656E5DAD-82F4-4AEB-BB43-73C9FA36DCD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19C913E0-7D12-4AEB-BF4D-C21572E863E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Monsters" sheetId="1" r:id="rId1"/>
@@ -208,7 +208,7 @@
             <family val="2"/>
             <scheme val="minor"/>
           </rPr>
-          <t>0-10. Low flees, ~5 wanders, high chases. Default 0.</t>
+          <t>Damage divisor in combat. 1 = full damage, 2 = half, etc. Default 1.</t>
         </r>
       </text>
     </comment>
@@ -222,7 +222,7 @@
             <family val="2"/>
             <scheme val="minor"/>
           </rPr>
-          <t>0-10. 0 never acts; any value above 0 gets one step per world round.</t>
+          <t>0-10. Low flees, ~5 wanders, high chases. Default 0.</t>
         </r>
       </text>
     </comment>
@@ -236,7 +236,7 @@
             <family val="2"/>
             <scheme val="minor"/>
           </rPr>
-          <t>0-10. Chance to stay still when idle/neutral = 1 - activeness/10.</t>
+          <t>0-10. 0 never acts; any value above 0 gets one step per world round.</t>
         </r>
       </text>
     </comment>
@@ -250,7 +250,7 @@
             <family val="2"/>
             <scheme val="minor"/>
           </rPr>
-          <t>Chebyshev vision distance in tiles. Default 20.</t>
+          <t>0-10. Chance to stay still when idle/neutral = 1 - activeness/10.</t>
         </r>
       </text>
     </comment>
@@ -264,7 +264,7 @@
             <family val="2"/>
             <scheme val="minor"/>
           </rPr>
-          <t>Comma-separated ability ids, or blank. Combat hooks not implemented yet.</t>
+          <t>Chebyshev vision distance in tiles. Default 20.</t>
         </r>
       </text>
     </comment>
@@ -278,7 +278,7 @@
             <family val="2"/>
             <scheme val="minor"/>
           </rPr>
-          <t>Leave blank for /static/monsters/sprites/{type_id}.png</t>
+          <t>Comma-separated ability ids, or blank. Combat hooks not implemented yet.</t>
         </r>
       </text>
     </comment>
@@ -292,7 +292,7 @@
             <family val="2"/>
             <scheme val="minor"/>
           </rPr>
-          <t>Leave blank for /static/monsters/portraits/{type_id}.png</t>
+          <t>Leave blank for /static/monsters/sprites/{type_id}.png</t>
         </r>
       </text>
     </comment>
@@ -306,11 +306,25 @@
             <family val="2"/>
             <scheme val="minor"/>
           </rPr>
+          <t>Leave blank for /static/monsters/portraits/{type_id}.png</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="U1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000015000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
           <t>Relative chance to appear when a monster spawns. 0 = never random-spawn.</t>
         </r>
       </text>
     </comment>
-    <comment ref="U1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000015000000}">
+    <comment ref="V1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000016000000}">
       <text>
         <r>
           <rPr>
@@ -329,7 +343,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="126">
   <si>
     <t>type_id</t>
   </si>
@@ -367,6 +381,9 @@
     <t>attack_power</t>
   </si>
   <si>
+    <t>armour</t>
+  </si>
+  <si>
     <t>aggression</t>
   </si>
   <si>
@@ -412,6 +429,162 @@
     <t>Current default spawn. Add more rows below.</t>
   </si>
   <si>
+    <t>skeleton</t>
+  </si>
+  <si>
+    <t>Skeleton</t>
+  </si>
+  <si>
+    <t>just a regular skeleton</t>
+  </si>
+  <si>
+    <t>/static/monsters/sprites/skeleton.png</t>
+  </si>
+  <si>
+    <t>/static/monsters/portraits/skeleton.png</t>
+  </si>
+  <si>
+    <t>ghost</t>
+  </si>
+  <si>
+    <t>Ghost</t>
+  </si>
+  <si>
+    <t>spoooky ghost</t>
+  </si>
+  <si>
+    <t>/static/monsters/sprites/ghost.png</t>
+  </si>
+  <si>
+    <t>/static/monsters/portraits/ghost.png</t>
+  </si>
+  <si>
+    <t>slime</t>
+  </si>
+  <si>
+    <t>Slime</t>
+  </si>
+  <si>
+    <t>/static/monsters/sprites/slime.png</t>
+  </si>
+  <si>
+    <t>/static/monsters/portraits/slime.png</t>
+  </si>
+  <si>
+    <t>ogre</t>
+  </si>
+  <si>
+    <t>Ogre</t>
+  </si>
+  <si>
+    <t>/static/monsters/sprites/ogre.png</t>
+  </si>
+  <si>
+    <t>/static/monsters/portraits/ogre.png</t>
+  </si>
+  <si>
+    <t>caveBat</t>
+  </si>
+  <si>
+    <t>Cave Bat</t>
+  </si>
+  <si>
+    <t>cave bat</t>
+  </si>
+  <si>
+    <t>/static/monsters/sprites/caveBat.png</t>
+  </si>
+  <si>
+    <t>/static/monsters/portraits/caveBat.png</t>
+  </si>
+  <si>
+    <t>giantRat</t>
+  </si>
+  <si>
+    <t>Giant Rat</t>
+  </si>
+  <si>
+    <t>giant rat</t>
+  </si>
+  <si>
+    <t>/static/monsters/sprites/giantRat.png</t>
+  </si>
+  <si>
+    <t>/static/monsters/portraits/giantRat.png</t>
+  </si>
+  <si>
+    <t>goblin</t>
+  </si>
+  <si>
+    <t>Goblin</t>
+  </si>
+  <si>
+    <t>/static/monsters/sprites/goblin.png</t>
+  </si>
+  <si>
+    <t>/static/monsters/portraits/goblin.png</t>
+  </si>
+  <si>
+    <t>poisonMushroom</t>
+  </si>
+  <si>
+    <t>Poison Mushroom</t>
+  </si>
+  <si>
+    <t>/static/monsters/sprites/poisonMushroom.png</t>
+  </si>
+  <si>
+    <t>/static/monsters/portraits/poisonMushroom.png</t>
+  </si>
+  <si>
+    <t>giantSnake</t>
+  </si>
+  <si>
+    <t>Giant Snake</t>
+  </si>
+  <si>
+    <t>/static/monsters/sprites/giantSnake.png</t>
+  </si>
+  <si>
+    <t>/static/monsters/portraits/giantSnake.png</t>
+  </si>
+  <si>
+    <t>imp</t>
+  </si>
+  <si>
+    <t>Imp</t>
+  </si>
+  <si>
+    <t>/static/monsters/sprites/imp.png</t>
+  </si>
+  <si>
+    <t>/static/monsters/portraits/imp.png</t>
+  </si>
+  <si>
+    <t>giantBeetle</t>
+  </si>
+  <si>
+    <t>Giant Beetle</t>
+  </si>
+  <si>
+    <t>/static/monsters/sprites/giantBeetle.png</t>
+  </si>
+  <si>
+    <t>/static/monsters/portraits/giantBeetle.png</t>
+  </si>
+  <si>
+    <t>mummy</t>
+  </si>
+  <si>
+    <t>Mummy</t>
+  </si>
+  <si>
+    <t>/static/monsters/sprites/mummy.png</t>
+  </si>
+  <si>
+    <t>/static/monsters/portraits/mummy.png</t>
+  </si>
+  <si>
     <t>How to use</t>
   </si>
   <si>
@@ -502,7 +675,10 @@
     <t>Max HP</t>
   </si>
   <si>
-    <t>Basic attack</t>
+    <t>Legacy; damage uses strength formula</t>
+  </si>
+  <si>
+    <t>Damage divisor. Default 1 (min 1)</t>
   </si>
   <si>
     <t>0-10 float</t>
@@ -545,169 +721,13 @@
   </si>
   <si>
     <t>Ignored on import</t>
-  </si>
-  <si>
-    <t>skeleton</t>
-  </si>
-  <si>
-    <t>Skeleton</t>
-  </si>
-  <si>
-    <t>/static/monsters/sprites/skeleton.png</t>
-  </si>
-  <si>
-    <t>/static/monsters/portraits/skeleton.png</t>
-  </si>
-  <si>
-    <t>just a regular skeleton</t>
-  </si>
-  <si>
-    <t>/static/monsters/sprites/ghost.png</t>
-  </si>
-  <si>
-    <t>/static/monsters/portraits/ghost.png</t>
-  </si>
-  <si>
-    <t>ghost</t>
-  </si>
-  <si>
-    <t>Ghost</t>
-  </si>
-  <si>
-    <t>spoooky ghost</t>
-  </si>
-  <si>
-    <t>slime</t>
-  </si>
-  <si>
-    <t>Slime</t>
-  </si>
-  <si>
-    <t>ogre</t>
-  </si>
-  <si>
-    <t>Ogre</t>
-  </si>
-  <si>
-    <t>/static/monsters/sprites/slime.png</t>
-  </si>
-  <si>
-    <t>/static/monsters/portraits/slime.png</t>
-  </si>
-  <si>
-    <t>/static/monsters/sprites/ogre.png</t>
-  </si>
-  <si>
-    <t>/static/monsters/portraits/ogre.png</t>
-  </si>
-  <si>
-    <t>caveBat</t>
-  </si>
-  <si>
-    <t>Cave Bat</t>
-  </si>
-  <si>
-    <t>cave bat</t>
-  </si>
-  <si>
-    <t>giantRat</t>
-  </si>
-  <si>
-    <t>Giant Rat</t>
-  </si>
-  <si>
-    <t>giant rat</t>
-  </si>
-  <si>
-    <t>/static/monsters/sprites/caveBat.png</t>
-  </si>
-  <si>
-    <t>/static/monsters/portraits/caveBat.png</t>
-  </si>
-  <si>
-    <t>/static/monsters/portraits/giantRat.png</t>
-  </si>
-  <si>
-    <t>/static/monsters/sprites/giantRat.png</t>
-  </si>
-  <si>
-    <t>goblin</t>
-  </si>
-  <si>
-    <t>Goblin</t>
-  </si>
-  <si>
-    <t>/static/monsters/sprites/goblin.png</t>
-  </si>
-  <si>
-    <t>/static/monsters/portraits/goblin.png</t>
-  </si>
-  <si>
-    <t>poisonMushroom</t>
-  </si>
-  <si>
-    <t>Poison Mushroom</t>
-  </si>
-  <si>
-    <t>/static/monsters/sprites/poisonMushroom.png</t>
-  </si>
-  <si>
-    <t>/static/monsters/portraits/poisonMushroom.png</t>
-  </si>
-  <si>
-    <t>giantSnake</t>
-  </si>
-  <si>
-    <t>Giant Snake</t>
-  </si>
-  <si>
-    <t>/static/monsters/sprites/giantSnake.png</t>
-  </si>
-  <si>
-    <t>/static/monsters/portraits/giantSnake.png</t>
-  </si>
-  <si>
-    <t>imp</t>
-  </si>
-  <si>
-    <t>Imp</t>
-  </si>
-  <si>
-    <t>/static/monsters/sprites/imp.png</t>
-  </si>
-  <si>
-    <t>/static/monsters/portraits/imp.png</t>
-  </si>
-  <si>
-    <t>giantBeetle</t>
-  </si>
-  <si>
-    <t>Giant Beetle</t>
-  </si>
-  <si>
-    <t>/static/monsters/sprites/giantBeetle.png</t>
-  </si>
-  <si>
-    <t>/static/monsters/portraits/giantBeetle.png</t>
-  </si>
-  <si>
-    <t>mummy</t>
-  </si>
-  <si>
-    <t>Mummy</t>
-  </si>
-  <si>
-    <t>/static/monsters/sprites/mummy.png</t>
-  </si>
-  <si>
-    <t>/static/monsters/portraits/mummy.png</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -733,8 +753,14 @@
       <color rgb="FF3D2B1F"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFF4E8D0"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -751,8 +777,13 @@
         <fgColor rgb="FFE6F4EA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF3D2B1F"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -775,11 +806,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFC4B8A8"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFC4B8A8"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFC4B8A8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFC4B8A8"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -797,6 +843,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1104,7 +1156,7 @@
   <sheetPr>
     <tabColor rgb="FF3D2B1F"/>
   </sheetPr>
-  <dimension ref="A1:U41"/>
+  <dimension ref="A1:V41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1114,8 +1166,7 @@
     <col min="5" max="10" width="10" customWidth="1"/>
     <col min="11" max="11" width="12" customWidth="1"/>
     <col min="12" max="12" width="14" customWidth="1"/>
-    <col min="13" max="13" width="12" customWidth="1"/>
-    <col min="14" max="14" width="10" customWidth="1"/>
+    <col min="13" max="14" width="10" customWidth="1"/>
     <col min="15" max="15" width="12" customWidth="1"/>
     <col min="16" max="16" width="13" customWidth="1"/>
     <col min="17" max="17" width="18" customWidth="1"/>
@@ -1125,7 +1176,7 @@
     <col min="21" max="21" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1162,7 +1213,7 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="9" t="s">
         <v>12</v>
       </c>
       <c r="N1" s="1" t="s">
@@ -1189,16 +1240,19 @@
       <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D2" s="2">
         <v>1</v>
@@ -1227,41 +1281,44 @@
       <c r="L2" s="2">
         <v>5</v>
       </c>
-      <c r="M2" s="2">
+      <c r="M2" s="10">
+        <v>1</v>
+      </c>
+      <c r="N2" s="2">
         <v>0</v>
       </c>
-      <c r="N2" s="2">
-        <v>10</v>
-      </c>
       <c r="O2" s="2">
+        <v>10</v>
+      </c>
+      <c r="P2" s="2">
         <v>2</v>
       </c>
-      <c r="P2" s="2">
+      <c r="Q2" s="2">
         <v>20</v>
       </c>
-      <c r="Q2" s="2"/>
-      <c r="R2" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="R2" s="2"/>
       <c r="S2" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="T2" s="2">
-        <v>1</v>
-      </c>
-      <c r="U2" s="2" t="s">
+      <c r="T2" s="2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="3" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+      <c r="U2" s="2">
+        <v>1</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>72</v>
+        <v>28</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>73</v>
+        <v>29</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>76</v>
+        <v>30</v>
       </c>
       <c r="D3" s="3">
         <v>1</v>
@@ -1290,41 +1347,44 @@
       <c r="L3" s="2">
         <v>10</v>
       </c>
-      <c r="M3" s="2">
+      <c r="M3" s="10">
+        <v>1</v>
+      </c>
+      <c r="N3" s="2">
         <v>0</v>
       </c>
-      <c r="N3" s="2">
-        <v>10</v>
-      </c>
       <c r="O3" s="2">
+        <v>10</v>
+      </c>
+      <c r="P3" s="2">
         <v>2</v>
       </c>
-      <c r="P3" s="2">
+      <c r="Q3" s="2">
         <v>20</v>
       </c>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2" t="s">
-        <v>74</v>
-      </c>
+      <c r="R3" s="2"/>
       <c r="S3" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="T3" s="2">
-        <v>1</v>
-      </c>
-      <c r="U3" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="U3" s="2">
+        <v>1</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>80</v>
+        <v>34</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="D4" s="3">
         <v>1</v>
@@ -1353,41 +1413,44 @@
       <c r="L4" s="2">
         <v>10</v>
       </c>
-      <c r="M4" s="2">
-        <v>10</v>
+      <c r="M4" s="10">
+        <v>1</v>
       </c>
       <c r="N4" s="2">
         <v>10</v>
       </c>
       <c r="O4" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="P4" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="2">
         <v>20</v>
       </c>
-      <c r="Q4" s="3"/>
-      <c r="R4" s="2" t="s">
-        <v>77</v>
-      </c>
+      <c r="R4" s="3"/>
       <c r="S4" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="T4" s="2">
-        <v>1</v>
-      </c>
-      <c r="U4" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+      <c r="T4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="U4" s="2">
+        <v>1</v>
+      </c>
+      <c r="V4" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>82</v>
+        <v>38</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>83</v>
+        <v>39</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>82</v>
+        <v>38</v>
       </c>
       <c r="D5" s="3">
         <v>1</v>
@@ -1416,41 +1479,44 @@
       <c r="L5" s="2">
         <v>10</v>
       </c>
-      <c r="M5" s="2">
+      <c r="M5" s="10">
+        <v>1</v>
+      </c>
+      <c r="N5" s="2">
         <v>5</v>
       </c>
-      <c r="N5" s="2">
-        <v>10</v>
-      </c>
       <c r="O5" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="P5" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q5" s="2">
         <v>20</v>
       </c>
-      <c r="Q5" s="3"/>
-      <c r="R5" s="2" t="s">
-        <v>86</v>
-      </c>
+      <c r="R5" s="3"/>
       <c r="S5" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="T5" s="2">
-        <v>1</v>
-      </c>
-      <c r="U5" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="6" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="T5" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="U5" s="2">
+        <v>1</v>
+      </c>
+      <c r="V5" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>84</v>
+        <v>42</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>85</v>
+        <v>43</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>84</v>
+        <v>42</v>
       </c>
       <c r="D6" s="3">
         <v>1</v>
@@ -1479,41 +1545,44 @@
       <c r="L6" s="2">
         <v>10</v>
       </c>
-      <c r="M6" s="2">
+      <c r="M6" s="10">
+        <v>1</v>
+      </c>
+      <c r="N6" s="2">
         <v>5</v>
       </c>
-      <c r="N6" s="2">
-        <v>10</v>
-      </c>
       <c r="O6" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="P6" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q6" s="2">
         <v>20</v>
       </c>
-      <c r="Q6" s="3"/>
-      <c r="R6" s="2" t="s">
-        <v>88</v>
-      </c>
+      <c r="R6" s="3"/>
       <c r="S6" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="T6" s="2">
-        <v>1</v>
-      </c>
-      <c r="U6" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="7" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+      <c r="T6" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="U6" s="2">
+        <v>1</v>
+      </c>
+      <c r="V6" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>90</v>
+        <v>46</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>91</v>
+        <v>47</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>92</v>
+        <v>48</v>
       </c>
       <c r="D7" s="3">
         <v>1</v>
@@ -1542,41 +1611,44 @@
       <c r="L7" s="2">
         <v>10</v>
       </c>
-      <c r="M7" s="2">
+      <c r="M7" s="10">
+        <v>1</v>
+      </c>
+      <c r="N7" s="2">
         <v>5</v>
       </c>
-      <c r="N7" s="2">
-        <v>10</v>
-      </c>
       <c r="O7" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="P7" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="2">
         <v>20</v>
       </c>
-      <c r="Q7" s="3"/>
-      <c r="R7" s="2" t="s">
-        <v>96</v>
-      </c>
+      <c r="R7" s="3"/>
       <c r="S7" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="T7" s="2">
-        <v>1</v>
-      </c>
-      <c r="U7" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="8" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+      <c r="T7" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="U7" s="2">
+        <v>1</v>
+      </c>
+      <c r="V7" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>93</v>
+        <v>51</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>94</v>
+        <v>52</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>95</v>
+        <v>53</v>
       </c>
       <c r="D8" s="3">
         <v>1</v>
@@ -1605,41 +1677,44 @@
       <c r="L8" s="2">
         <v>10</v>
       </c>
-      <c r="M8" s="2">
+      <c r="M8" s="10">
+        <v>1</v>
+      </c>
+      <c r="N8" s="2">
         <v>5</v>
       </c>
-      <c r="N8" s="2">
-        <v>10</v>
-      </c>
       <c r="O8" s="2">
         <v>10</v>
       </c>
       <c r="P8" s="2">
+        <v>10</v>
+      </c>
+      <c r="Q8" s="2">
         <v>20</v>
       </c>
-      <c r="Q8" s="3"/>
-      <c r="R8" s="2" t="s">
-        <v>99</v>
-      </c>
+      <c r="R8" s="3"/>
       <c r="S8" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="T8" s="2">
-        <v>1</v>
-      </c>
-      <c r="U8" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+      <c r="T8" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="U8" s="2">
+        <v>1</v>
+      </c>
+      <c r="V8" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>100</v>
+        <v>56</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>101</v>
+        <v>57</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>101</v>
+        <v>57</v>
       </c>
       <c r="D9" s="3">
         <v>1</v>
@@ -1668,41 +1743,44 @@
       <c r="L9" s="2">
         <v>10</v>
       </c>
-      <c r="M9" s="2">
+      <c r="M9" s="10">
+        <v>1</v>
+      </c>
+      <c r="N9" s="2">
         <v>5</v>
       </c>
-      <c r="N9" s="2">
-        <v>10</v>
-      </c>
       <c r="O9" s="2">
+        <v>10</v>
+      </c>
+      <c r="P9" s="2">
         <v>5</v>
       </c>
-      <c r="P9" s="2">
+      <c r="Q9" s="2">
         <v>20</v>
       </c>
-      <c r="Q9" s="3"/>
-      <c r="R9" s="2" t="s">
-        <v>102</v>
-      </c>
+      <c r="R9" s="3"/>
       <c r="S9" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="T9" s="2">
-        <v>1</v>
-      </c>
-      <c r="U9" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+      <c r="T9" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="U9" s="2">
+        <v>1</v>
+      </c>
+      <c r="V9" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>104</v>
+        <v>60</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>105</v>
+        <v>61</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>105</v>
+        <v>61</v>
       </c>
       <c r="D10" s="3">
         <v>1</v>
@@ -1731,41 +1809,44 @@
       <c r="L10" s="2">
         <v>10</v>
       </c>
-      <c r="M10" s="2">
+      <c r="M10" s="10">
+        <v>1</v>
+      </c>
+      <c r="N10" s="2">
         <v>5</v>
       </c>
-      <c r="N10" s="2">
-        <v>10</v>
-      </c>
       <c r="O10" s="2">
+        <v>10</v>
+      </c>
+      <c r="P10" s="2">
         <v>4</v>
       </c>
-      <c r="P10" s="2">
+      <c r="Q10" s="2">
         <v>20</v>
       </c>
-      <c r="Q10" s="3"/>
-      <c r="R10" s="2" t="s">
-        <v>106</v>
-      </c>
+      <c r="R10" s="3"/>
       <c r="S10" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="T10" s="2">
-        <v>1</v>
-      </c>
-      <c r="U10" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="11" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+      <c r="T10" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="U10" s="2">
+        <v>1</v>
+      </c>
+      <c r="V10" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>108</v>
+        <v>64</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>109</v>
+        <v>65</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>109</v>
+        <v>65</v>
       </c>
       <c r="D11" s="3">
         <v>1</v>
@@ -1794,41 +1875,44 @@
       <c r="L11" s="2">
         <v>10</v>
       </c>
-      <c r="M11" s="2">
+      <c r="M11" s="10">
+        <v>1</v>
+      </c>
+      <c r="N11" s="2">
         <v>5</v>
       </c>
-      <c r="N11" s="2">
-        <v>10</v>
-      </c>
       <c r="O11" s="2">
         <v>10</v>
       </c>
       <c r="P11" s="2">
+        <v>10</v>
+      </c>
+      <c r="Q11" s="2">
         <v>20</v>
       </c>
-      <c r="Q11" s="3"/>
-      <c r="R11" s="2" t="s">
-        <v>110</v>
-      </c>
+      <c r="R11" s="3"/>
       <c r="S11" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="T11" s="2">
-        <v>1</v>
-      </c>
-      <c r="U11" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="12" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+      <c r="T11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="U11" s="2">
+        <v>1</v>
+      </c>
+      <c r="V11" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>112</v>
+        <v>68</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>113</v>
+        <v>69</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>113</v>
+        <v>69</v>
       </c>
       <c r="D12" s="3">
         <v>1</v>
@@ -1857,41 +1941,44 @@
       <c r="L12" s="2">
         <v>10</v>
       </c>
-      <c r="M12" s="2">
+      <c r="M12" s="10">
+        <v>1</v>
+      </c>
+      <c r="N12" s="2">
         <v>5</v>
       </c>
-      <c r="N12" s="2">
-        <v>10</v>
-      </c>
       <c r="O12" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="P12" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q12" s="2">
         <v>20</v>
       </c>
-      <c r="Q12" s="3"/>
-      <c r="R12" s="2" t="s">
-        <v>114</v>
-      </c>
+      <c r="R12" s="3"/>
       <c r="S12" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="T12" s="2">
-        <v>1</v>
-      </c>
-      <c r="U12" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="13" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+      <c r="T12" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="U12" s="2">
+        <v>1</v>
+      </c>
+      <c r="V12" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>116</v>
+        <v>72</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>117</v>
+        <v>73</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>117</v>
+        <v>73</v>
       </c>
       <c r="D13" s="3">
         <v>1</v>
@@ -1920,41 +2007,44 @@
       <c r="L13" s="2">
         <v>10</v>
       </c>
-      <c r="M13" s="2">
+      <c r="M13" s="10">
+        <v>6</v>
+      </c>
+      <c r="N13" s="2">
         <v>5</v>
       </c>
-      <c r="N13" s="2">
-        <v>10</v>
-      </c>
       <c r="O13" s="2">
         <v>10</v>
       </c>
       <c r="P13" s="2">
+        <v>10</v>
+      </c>
+      <c r="Q13" s="2">
         <v>20</v>
       </c>
-      <c r="Q13" s="3"/>
-      <c r="R13" s="2" t="s">
-        <v>118</v>
-      </c>
+      <c r="R13" s="3"/>
       <c r="S13" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="T13" s="2">
-        <v>1</v>
-      </c>
-      <c r="U13" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="14" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+      <c r="T13" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="U13" s="2">
+        <v>1</v>
+      </c>
+      <c r="V13" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>120</v>
+        <v>76</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>121</v>
+        <v>77</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>121</v>
+        <v>77</v>
       </c>
       <c r="D14" s="3">
         <v>1</v>
@@ -1983,33 +2073,36 @@
       <c r="L14" s="2">
         <v>10</v>
       </c>
-      <c r="M14" s="2">
+      <c r="M14" s="10">
+        <v>1</v>
+      </c>
+      <c r="N14" s="2">
         <v>5</v>
       </c>
-      <c r="N14" s="2">
-        <v>10</v>
-      </c>
       <c r="O14" s="2">
         <v>10</v>
       </c>
       <c r="P14" s="2">
+        <v>10</v>
+      </c>
+      <c r="Q14" s="2">
         <v>20</v>
       </c>
-      <c r="Q14" s="3"/>
-      <c r="R14" s="2" t="s">
-        <v>122</v>
-      </c>
+      <c r="R14" s="3"/>
       <c r="S14" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="T14" s="2">
-        <v>1</v>
-      </c>
-      <c r="U14" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+      <c r="T14" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="U14" s="2">
+        <v>1</v>
+      </c>
+      <c r="V14" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -2022,7 +2115,6 @@
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
       <c r="L15" s="3"/>
-      <c r="M15" s="3"/>
       <c r="N15" s="3"/>
       <c r="O15" s="3"/>
       <c r="P15" s="3"/>
@@ -2031,8 +2123,9 @@
       <c r="S15" s="3"/>
       <c r="T15" s="3"/>
       <c r="U15" s="3"/>
-    </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V15" s="3"/>
+    </row>
+    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -2045,7 +2138,6 @@
       <c r="J16" s="3"/>
       <c r="K16" s="3"/>
       <c r="L16" s="3"/>
-      <c r="M16" s="3"/>
       <c r="N16" s="3"/>
       <c r="O16" s="3"/>
       <c r="P16" s="3"/>
@@ -2054,8 +2146,9 @@
       <c r="S16" s="3"/>
       <c r="T16" s="3"/>
       <c r="U16" s="3"/>
-    </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V16" s="3"/>
+    </row>
+    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -2068,7 +2161,6 @@
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
       <c r="L17" s="3"/>
-      <c r="M17" s="3"/>
       <c r="N17" s="3"/>
       <c r="O17" s="3"/>
       <c r="P17" s="3"/>
@@ -2077,8 +2169,9 @@
       <c r="S17" s="3"/>
       <c r="T17" s="3"/>
       <c r="U17" s="3"/>
-    </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V17" s="3"/>
+    </row>
+    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -2091,7 +2184,6 @@
       <c r="J18" s="3"/>
       <c r="K18" s="3"/>
       <c r="L18" s="3"/>
-      <c r="M18" s="3"/>
       <c r="N18" s="3"/>
       <c r="O18" s="3"/>
       <c r="P18" s="3"/>
@@ -2100,8 +2192,9 @@
       <c r="S18" s="3"/>
       <c r="T18" s="3"/>
       <c r="U18" s="3"/>
-    </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V18" s="3"/>
+    </row>
+    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -2114,7 +2207,6 @@
       <c r="J19" s="3"/>
       <c r="K19" s="3"/>
       <c r="L19" s="3"/>
-      <c r="M19" s="3"/>
       <c r="N19" s="3"/>
       <c r="O19" s="3"/>
       <c r="P19" s="3"/>
@@ -2123,8 +2215,9 @@
       <c r="S19" s="3"/>
       <c r="T19" s="3"/>
       <c r="U19" s="3"/>
-    </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V19" s="3"/>
+    </row>
+    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -2137,7 +2230,6 @@
       <c r="J20" s="3"/>
       <c r="K20" s="3"/>
       <c r="L20" s="3"/>
-      <c r="M20" s="3"/>
       <c r="N20" s="3"/>
       <c r="O20" s="3"/>
       <c r="P20" s="3"/>
@@ -2146,8 +2238,9 @@
       <c r="S20" s="3"/>
       <c r="T20" s="3"/>
       <c r="U20" s="3"/>
-    </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V20" s="3"/>
+    </row>
+    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
@@ -2160,7 +2253,6 @@
       <c r="J21" s="3"/>
       <c r="K21" s="3"/>
       <c r="L21" s="3"/>
-      <c r="M21" s="3"/>
       <c r="N21" s="3"/>
       <c r="O21" s="3"/>
       <c r="P21" s="3"/>
@@ -2169,8 +2261,9 @@
       <c r="S21" s="3"/>
       <c r="T21" s="3"/>
       <c r="U21" s="3"/>
-    </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V21" s="3"/>
+    </row>
+    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
@@ -2183,7 +2276,6 @@
       <c r="J22" s="3"/>
       <c r="K22" s="3"/>
       <c r="L22" s="3"/>
-      <c r="M22" s="3"/>
       <c r="N22" s="3"/>
       <c r="O22" s="3"/>
       <c r="P22" s="3"/>
@@ -2192,8 +2284,9 @@
       <c r="S22" s="3"/>
       <c r="T22" s="3"/>
       <c r="U22" s="3"/>
-    </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V22" s="3"/>
+    </row>
+    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -2206,7 +2299,6 @@
       <c r="J23" s="3"/>
       <c r="K23" s="3"/>
       <c r="L23" s="3"/>
-      <c r="M23" s="3"/>
       <c r="N23" s="3"/>
       <c r="O23" s="3"/>
       <c r="P23" s="3"/>
@@ -2215,8 +2307,9 @@
       <c r="S23" s="3"/>
       <c r="T23" s="3"/>
       <c r="U23" s="3"/>
-    </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V23" s="3"/>
+    </row>
+    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -2229,7 +2322,6 @@
       <c r="J24" s="3"/>
       <c r="K24" s="3"/>
       <c r="L24" s="3"/>
-      <c r="M24" s="3"/>
       <c r="N24" s="3"/>
       <c r="O24" s="3"/>
       <c r="P24" s="3"/>
@@ -2238,8 +2330,9 @@
       <c r="S24" s="3"/>
       <c r="T24" s="3"/>
       <c r="U24" s="3"/>
-    </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V24" s="3"/>
+    </row>
+    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -2252,7 +2345,6 @@
       <c r="J25" s="3"/>
       <c r="K25" s="3"/>
       <c r="L25" s="3"/>
-      <c r="M25" s="3"/>
       <c r="N25" s="3"/>
       <c r="O25" s="3"/>
       <c r="P25" s="3"/>
@@ -2261,8 +2353,9 @@
       <c r="S25" s="3"/>
       <c r="T25" s="3"/>
       <c r="U25" s="3"/>
-    </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V25" s="3"/>
+    </row>
+    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
@@ -2275,7 +2368,6 @@
       <c r="J26" s="3"/>
       <c r="K26" s="3"/>
       <c r="L26" s="3"/>
-      <c r="M26" s="3"/>
       <c r="N26" s="3"/>
       <c r="O26" s="3"/>
       <c r="P26" s="3"/>
@@ -2284,8 +2376,9 @@
       <c r="S26" s="3"/>
       <c r="T26" s="3"/>
       <c r="U26" s="3"/>
-    </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V26" s="3"/>
+    </row>
+    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -2298,7 +2391,6 @@
       <c r="J27" s="3"/>
       <c r="K27" s="3"/>
       <c r="L27" s="3"/>
-      <c r="M27" s="3"/>
       <c r="N27" s="3"/>
       <c r="O27" s="3"/>
       <c r="P27" s="3"/>
@@ -2307,8 +2399,9 @@
       <c r="S27" s="3"/>
       <c r="T27" s="3"/>
       <c r="U27" s="3"/>
-    </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V27" s="3"/>
+    </row>
+    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -2321,7 +2414,6 @@
       <c r="J28" s="3"/>
       <c r="K28" s="3"/>
       <c r="L28" s="3"/>
-      <c r="M28" s="3"/>
       <c r="N28" s="3"/>
       <c r="O28" s="3"/>
       <c r="P28" s="3"/>
@@ -2330,8 +2422,9 @@
       <c r="S28" s="3"/>
       <c r="T28" s="3"/>
       <c r="U28" s="3"/>
-    </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V28" s="3"/>
+    </row>
+    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -2344,7 +2437,6 @@
       <c r="J29" s="3"/>
       <c r="K29" s="3"/>
       <c r="L29" s="3"/>
-      <c r="M29" s="3"/>
       <c r="N29" s="3"/>
       <c r="O29" s="3"/>
       <c r="P29" s="3"/>
@@ -2353,8 +2445,9 @@
       <c r="S29" s="3"/>
       <c r="T29" s="3"/>
       <c r="U29" s="3"/>
-    </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V29" s="3"/>
+    </row>
+    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
@@ -2367,7 +2460,6 @@
       <c r="J30" s="3"/>
       <c r="K30" s="3"/>
       <c r="L30" s="3"/>
-      <c r="M30" s="3"/>
       <c r="N30" s="3"/>
       <c r="O30" s="3"/>
       <c r="P30" s="3"/>
@@ -2376,8 +2468,9 @@
       <c r="S30" s="3"/>
       <c r="T30" s="3"/>
       <c r="U30" s="3"/>
-    </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V30" s="3"/>
+    </row>
+    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
@@ -2390,7 +2483,6 @@
       <c r="J31" s="3"/>
       <c r="K31" s="3"/>
       <c r="L31" s="3"/>
-      <c r="M31" s="3"/>
       <c r="N31" s="3"/>
       <c r="O31" s="3"/>
       <c r="P31" s="3"/>
@@ -2399,8 +2491,9 @@
       <c r="S31" s="3"/>
       <c r="T31" s="3"/>
       <c r="U31" s="3"/>
-    </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V31" s="3"/>
+    </row>
+    <row r="32" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
@@ -2413,7 +2506,6 @@
       <c r="J32" s="3"/>
       <c r="K32" s="3"/>
       <c r="L32" s="3"/>
-      <c r="M32" s="3"/>
       <c r="N32" s="3"/>
       <c r="O32" s="3"/>
       <c r="P32" s="3"/>
@@ -2422,8 +2514,9 @@
       <c r="S32" s="3"/>
       <c r="T32" s="3"/>
       <c r="U32" s="3"/>
-    </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V32" s="3"/>
+    </row>
+    <row r="33" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
@@ -2436,7 +2529,6 @@
       <c r="J33" s="3"/>
       <c r="K33" s="3"/>
       <c r="L33" s="3"/>
-      <c r="M33" s="3"/>
       <c r="N33" s="3"/>
       <c r="O33" s="3"/>
       <c r="P33" s="3"/>
@@ -2445,8 +2537,9 @@
       <c r="S33" s="3"/>
       <c r="T33" s="3"/>
       <c r="U33" s="3"/>
-    </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V33" s="3"/>
+    </row>
+    <row r="34" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
@@ -2459,7 +2552,6 @@
       <c r="J34" s="3"/>
       <c r="K34" s="3"/>
       <c r="L34" s="3"/>
-      <c r="M34" s="3"/>
       <c r="N34" s="3"/>
       <c r="O34" s="3"/>
       <c r="P34" s="3"/>
@@ -2468,8 +2560,9 @@
       <c r="S34" s="3"/>
       <c r="T34" s="3"/>
       <c r="U34" s="3"/>
-    </row>
-    <row r="35" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V34" s="3"/>
+    </row>
+    <row r="35" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A35" s="3"/>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
@@ -2482,7 +2575,6 @@
       <c r="J35" s="3"/>
       <c r="K35" s="3"/>
       <c r="L35" s="3"/>
-      <c r="M35" s="3"/>
       <c r="N35" s="3"/>
       <c r="O35" s="3"/>
       <c r="P35" s="3"/>
@@ -2491,8 +2583,9 @@
       <c r="S35" s="3"/>
       <c r="T35" s="3"/>
       <c r="U35" s="3"/>
-    </row>
-    <row r="36" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V35" s="3"/>
+    </row>
+    <row r="36" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A36" s="3"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
@@ -2505,7 +2598,6 @@
       <c r="J36" s="3"/>
       <c r="K36" s="3"/>
       <c r="L36" s="3"/>
-      <c r="M36" s="3"/>
       <c r="N36" s="3"/>
       <c r="O36" s="3"/>
       <c r="P36" s="3"/>
@@ -2514,8 +2606,9 @@
       <c r="S36" s="3"/>
       <c r="T36" s="3"/>
       <c r="U36" s="3"/>
-    </row>
-    <row r="37" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V36" s="3"/>
+    </row>
+    <row r="37" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A37" s="3"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
@@ -2528,7 +2621,6 @@
       <c r="J37" s="3"/>
       <c r="K37" s="3"/>
       <c r="L37" s="3"/>
-      <c r="M37" s="3"/>
       <c r="N37" s="3"/>
       <c r="O37" s="3"/>
       <c r="P37" s="3"/>
@@ -2537,8 +2629,9 @@
       <c r="S37" s="3"/>
       <c r="T37" s="3"/>
       <c r="U37" s="3"/>
-    </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V37" s="3"/>
+    </row>
+    <row r="38" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A38" s="3"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
@@ -2551,7 +2644,6 @@
       <c r="J38" s="3"/>
       <c r="K38" s="3"/>
       <c r="L38" s="3"/>
-      <c r="M38" s="3"/>
       <c r="N38" s="3"/>
       <c r="O38" s="3"/>
       <c r="P38" s="3"/>
@@ -2560,8 +2652,9 @@
       <c r="S38" s="3"/>
       <c r="T38" s="3"/>
       <c r="U38" s="3"/>
-    </row>
-    <row r="39" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V38" s="3"/>
+    </row>
+    <row r="39" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A39" s="3"/>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
@@ -2574,7 +2667,6 @@
       <c r="J39" s="3"/>
       <c r="K39" s="3"/>
       <c r="L39" s="3"/>
-      <c r="M39" s="3"/>
       <c r="N39" s="3"/>
       <c r="O39" s="3"/>
       <c r="P39" s="3"/>
@@ -2583,8 +2675,9 @@
       <c r="S39" s="3"/>
       <c r="T39" s="3"/>
       <c r="U39" s="3"/>
-    </row>
-    <row r="40" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V39" s="3"/>
+    </row>
+    <row r="40" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A40" s="3"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
@@ -2597,7 +2690,6 @@
       <c r="J40" s="3"/>
       <c r="K40" s="3"/>
       <c r="L40" s="3"/>
-      <c r="M40" s="3"/>
       <c r="N40" s="3"/>
       <c r="O40" s="3"/>
       <c r="P40" s="3"/>
@@ -2606,8 +2698,9 @@
       <c r="S40" s="3"/>
       <c r="T40" s="3"/>
       <c r="U40" s="3"/>
-    </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V40" s="3"/>
+    </row>
+    <row r="41" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A41" s="3"/>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
@@ -2620,7 +2713,6 @@
       <c r="J41" s="3"/>
       <c r="K41" s="3"/>
       <c r="L41" s="3"/>
-      <c r="M41" s="3"/>
       <c r="N41" s="3"/>
       <c r="O41" s="3"/>
       <c r="P41" s="3"/>
@@ -2629,6 +2721,7 @@
       <c r="S41" s="3"/>
       <c r="T41" s="3"/>
       <c r="U41" s="3"/>
+      <c r="V41" s="3"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U41" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
@@ -2645,9 +2738,9 @@
     <col min="1" max="1" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>27</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -2655,83 +2748,83 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>28</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>29</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>30</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>31</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>32</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>33</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>34</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="5"/>
     </row>
-    <row r="11" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>35</v>
+        <v>88</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>36</v>
+        <v>89</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>37</v>
+        <v>90</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>38</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>39</v>
+        <v>92</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="5"/>
     </row>
-    <row r="17" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>40</v>
+        <v>93</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>41</v>
+        <v>94</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>42</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -2741,7 +2834,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -2752,16 +2845,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>43</v>
+        <v>96</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>44</v>
+        <v>97</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>45</v>
+        <v>98</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>46</v>
+        <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -2769,13 +2862,13 @@
         <v>0</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>47</v>
+        <v>100</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>48</v>
+        <v>101</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>49</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -2783,13 +2876,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>47</v>
+        <v>100</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>48</v>
+        <v>101</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>50</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -2797,13 +2890,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>48</v>
+        <v>101</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>52</v>
+        <v>105</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -2811,27 +2904,27 @@
         <v>3</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>5</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>53</v>
+        <v>106</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>47</v>
+        <v>100</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>55</v>
+        <v>108</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -2839,13 +2932,13 @@
         <v>10</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>47</v>
+        <v>100</v>
       </c>
       <c r="C7" s="8" t="s">
         <v>5</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>56</v>
+        <v>109</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -2853,27 +2946,27 @@
         <v>11</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>47</v>
+        <v>104</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>5</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>57</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>59</v>
+      <c r="B9" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -2881,13 +2974,13 @@
         <v>13</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>58</v>
+        <v>112</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>60</v>
+        <v>113</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -2895,13 +2988,13 @@
         <v>14</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>58</v>
+        <v>112</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>61</v>
+        <v>114</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -2909,13 +3002,13 @@
         <v>15</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>5</v>
+        <v>112</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>62</v>
+        <v>115</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -2923,13 +3016,13 @@
         <v>16</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>63</v>
+        <v>5</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>64</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -2937,13 +3030,13 @@
         <v>17</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>65</v>
+        <v>117</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>66</v>
+        <v>118</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -2951,13 +3044,13 @@
         <v>18</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>65</v>
+        <v>119</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>67</v>
+        <v>120</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -2965,13 +3058,13 @@
         <v>19</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>68</v>
+        <v>119</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>69</v>
+        <v>121</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -2979,13 +3072,27 @@
         <v>20</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>70</v>
+        <v>122</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>71</v>
+        <v>123</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enhance monster attributes with agility and combat logic adjustments
- Introduced an `agility` attribute to the `MonsterTypeDef` class, allowing for more nuanced combat interactions.
- Updated the `Monster` class to incorporate the `agility` attribute in combat calculations, influencing evasion and attack success rates.
- Modified related documentation and test cases to reflect the addition of the `agility` attribute, ensuring clarity and consistency across the codebase.
</commit_message>
<xml_diff>
--- a/monster_types.xlsx
+++ b/monster_types.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\info\Documents\Projects\dungeon-console\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{378D68F6-A9FD-4D9D-835F-BA2140164527}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48F23979-A964-4AEE-9B57-D215E1827005}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Monsters" sheetId="1" r:id="rId1"/>
@@ -1522,7 +1522,7 @@
         <v>6</v>
       </c>
       <c r="G5" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H5" s="8">
         <v>3</v>

</xml_diff>

<commit_message>
Refactor monster attributes to include critical hit mechanics and adjust combat logic
- Introduced a `critical_hit_chance` attribute to the `MonsterTypeDef` class, enhancing combat dynamics.
- Updated the `Monster` class to incorporate the `critical_hit_chance` in damage calculations, affecting overall combat outcomes.
- Modified related documentation and test cases to reflect the addition of the `critical_hit_chance` attribute, ensuring clarity and consistency across the codebase.
</commit_message>
<xml_diff>
--- a/monster_types.xlsx
+++ b/monster_types.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\info\Documents\Projects\dungeon-console\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48F23979-A964-4AEE-9B57-D215E1827005}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD3F1ECF-5936-4B44-BE02-B2BB2303866E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,20 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Monsters!$A$1:$W$41</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 

</xml_diff>

<commit_message>
Refactor combat system for improved player feedback and interaction
- Enhanced combat status messages to provide clearer information about player actions and outcomes.
- Streamlined combatant selection processes to improve user experience during battles.
- Updated event handling for combat interactions, allowing for more intuitive target selection.
- Improved feedback mechanisms for monster interactions to ensure unique identification and better player notifications.
- Refactored combat update processes to maintain game flow and clarity during encounters.
</commit_message>
<xml_diff>
--- a/monster_types.xlsx
+++ b/monster_types.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\info\Documents\Projects\dungeon-console\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D95AC6D-573A-4F53-8F73-C0022221775E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46280EB6-5833-4E9E-8C40-6475C00C3B25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1381,7 +1381,7 @@
         <v>28</v>
       </c>
       <c r="W2" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X2" s="8" t="s">
         <v>29</v>
@@ -1453,7 +1453,7 @@
         <v>34</v>
       </c>
       <c r="W3" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X3" s="8" t="s">
         <v>29</v>
@@ -1525,7 +1525,7 @@
         <v>39</v>
       </c>
       <c r="W4" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X4" s="8" t="s">
         <v>29</v>
@@ -1597,7 +1597,7 @@
         <v>43</v>
       </c>
       <c r="W5" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X5" s="8" t="s">
         <v>29</v>
@@ -1669,7 +1669,7 @@
         <v>47</v>
       </c>
       <c r="W6" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X6" s="8" t="s">
         <v>29</v>
@@ -1741,7 +1741,7 @@
         <v>52</v>
       </c>
       <c r="W7" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X7" s="8" t="s">
         <v>29</v>
@@ -1885,7 +1885,7 @@
         <v>61</v>
       </c>
       <c r="W9" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X9" s="8" t="s">
         <v>29</v>
@@ -1957,7 +1957,7 @@
         <v>65</v>
       </c>
       <c r="W10" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X10" s="8" t="s">
         <v>29</v>
@@ -2029,7 +2029,7 @@
         <v>69</v>
       </c>
       <c r="W11" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X11" s="8" t="s">
         <v>29</v>
@@ -2101,7 +2101,7 @@
         <v>73</v>
       </c>
       <c r="W12" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X12" s="8" t="s">
         <v>29</v>
@@ -2173,7 +2173,7 @@
         <v>77</v>
       </c>
       <c r="W13" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X13" s="8" t="s">
         <v>29</v>
@@ -2245,7 +2245,7 @@
         <v>81</v>
       </c>
       <c r="W14" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X14" s="8" t="s">
         <v>29</v>

</xml_diff>

<commit_message>
Refactor player save data handling and world persistence management
- Updated player save data structure to include additional attributes for enhanced gameplay continuity.
- Improved logic for restoring player states from saved world data, ensuring a seamless experience.
- Enhanced GameState class to better manage world persistence and track changes effectively.
- Refined socket communication to handle player death events and update the UI accordingly.
- Adjusted database configuration to support the new world persistence features.
</commit_message>
<xml_diff>
--- a/monster_types.xlsx
+++ b/monster_types.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\info\Documents\Projects\dungeon-console\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46280EB6-5833-4E9E-8C40-6475C00C3B25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66B0DB2A-AC09-442B-BE7E-6FC939E71351}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1381,7 +1381,7 @@
         <v>28</v>
       </c>
       <c r="W2" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X2" s="8" t="s">
         <v>29</v>
@@ -1453,7 +1453,7 @@
         <v>34</v>
       </c>
       <c r="W3" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X3" s="8" t="s">
         <v>29</v>
@@ -1525,7 +1525,7 @@
         <v>39</v>
       </c>
       <c r="W4" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X4" s="8" t="s">
         <v>29</v>
@@ -1597,7 +1597,7 @@
         <v>43</v>
       </c>
       <c r="W5" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X5" s="8" t="s">
         <v>29</v>
@@ -1669,7 +1669,7 @@
         <v>47</v>
       </c>
       <c r="W6" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X6" s="8" t="s">
         <v>29</v>
@@ -1741,7 +1741,7 @@
         <v>52</v>
       </c>
       <c r="W7" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X7" s="8" t="s">
         <v>29</v>
@@ -1885,7 +1885,7 @@
         <v>61</v>
       </c>
       <c r="W9" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X9" s="8" t="s">
         <v>29</v>
@@ -1957,7 +1957,7 @@
         <v>65</v>
       </c>
       <c r="W10" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X10" s="8" t="s">
         <v>29</v>
@@ -2029,7 +2029,7 @@
         <v>69</v>
       </c>
       <c r="W11" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X11" s="8" t="s">
         <v>29</v>
@@ -2101,7 +2101,7 @@
         <v>73</v>
       </c>
       <c r="W12" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X12" s="8" t="s">
         <v>29</v>
@@ -2173,7 +2173,7 @@
         <v>77</v>
       </c>
       <c r="W13" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X13" s="8" t="s">
         <v>29</v>
@@ -2245,7 +2245,7 @@
         <v>81</v>
       </c>
       <c r="W14" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X14" s="8" t="s">
         <v>29</v>

</xml_diff>

<commit_message>
Update monster sheet and regenerate Elo ladder ratings.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/monster_types.xlsx
+++ b/monster_types.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\info\Documents\Projects\dungeon-console\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66B0DB2A-AC09-442B-BE7E-6FC939E71351}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1BC4C52-7CEA-4BF8-B7EB-9DF0DD0CD82F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,20 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Monsters!$A$1:$W$41</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1227,9 +1240,7 @@
     <col min="3" max="3" width="42" customWidth="1"/>
     <col min="4" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="12" width="10" customWidth="1"/>
-    <col min="13" max="13" width="12" customWidth="1"/>
-    <col min="14" max="14" width="10" customWidth="1"/>
+    <col min="7" max="14" width="10" customWidth="1"/>
     <col min="15" max="15" width="12" customWidth="1"/>
     <col min="16" max="16" width="10" customWidth="1"/>
     <col min="17" max="17" width="12" customWidth="1"/>
@@ -1278,7 +1289,7 @@
       <c r="L1" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="7" t="s">
         <v>12</v>
       </c>
       <c r="N1" s="7" t="s">
@@ -1332,28 +1343,28 @@
         <v>10</v>
       </c>
       <c r="F2" s="8">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G2" s="8">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H2" s="8">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="I2" s="8">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="J2" s="8">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="K2" s="8">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="L2" s="8">
-        <v>4</v>
-      </c>
-      <c r="M2">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="M2" s="8">
+        <v>12</v>
       </c>
       <c r="N2" s="8">
         <v>16</v>
@@ -1407,25 +1418,25 @@
         <v>6</v>
       </c>
       <c r="G3" s="8">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H3" s="8">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="I3" s="8">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="J3" s="8">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="K3" s="8">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="L3" s="8">
-        <v>4</v>
-      </c>
-      <c r="M3">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="M3" s="8">
+        <v>12</v>
       </c>
       <c r="N3" s="8">
         <v>10</v>
@@ -1479,25 +1490,25 @@
         <v>6</v>
       </c>
       <c r="G4" s="8">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H4" s="8">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="I4" s="8">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="J4" s="8">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="K4" s="8">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="L4" s="8">
-        <v>4</v>
-      </c>
-      <c r="M4">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="M4" s="8">
+        <v>15</v>
       </c>
       <c r="N4" s="8">
         <v>20</v>
@@ -1551,25 +1562,25 @@
         <v>6</v>
       </c>
       <c r="G5" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H5" s="8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I5" s="8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J5" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K5" s="8">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L5" s="8">
-        <v>4</v>
-      </c>
-      <c r="M5">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="M5" s="8">
+        <v>5</v>
       </c>
       <c r="N5" s="8">
         <v>20</v>
@@ -1620,28 +1631,28 @@
         <v>10</v>
       </c>
       <c r="F6" s="8">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G6" s="8">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="H6" s="8">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="I6" s="8">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="J6" s="8">
+        <v>8</v>
+      </c>
+      <c r="K6" s="8">
         <v>2</v>
       </c>
-      <c r="K6" s="8">
-        <v>4</v>
-      </c>
       <c r="L6" s="8">
-        <v>4</v>
-      </c>
-      <c r="M6">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="M6" s="8">
+        <v>10</v>
       </c>
       <c r="N6" s="8">
         <v>20</v>
@@ -1695,25 +1706,25 @@
         <v>6</v>
       </c>
       <c r="G7" s="8">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="H7" s="8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I7" s="8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J7" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K7" s="8">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L7" s="8">
-        <v>4</v>
-      </c>
-      <c r="M7">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="M7" s="8">
+        <v>10</v>
       </c>
       <c r="N7" s="8">
         <v>20</v>
@@ -1767,25 +1778,25 @@
         <v>6</v>
       </c>
       <c r="G8" s="8">
+        <v>2</v>
+      </c>
+      <c r="H8" s="8">
+        <v>4</v>
+      </c>
+      <c r="I8" s="8">
+        <v>4</v>
+      </c>
+      <c r="J8" s="8">
+        <v>1</v>
+      </c>
+      <c r="K8" s="8">
+        <v>15</v>
+      </c>
+      <c r="L8" s="8">
         <v>5</v>
       </c>
-      <c r="H8" s="8">
-        <v>3</v>
-      </c>
-      <c r="I8" s="8">
-        <v>3</v>
-      </c>
-      <c r="J8" s="8">
-        <v>2</v>
-      </c>
-      <c r="K8" s="8">
-        <v>4</v>
-      </c>
-      <c r="L8" s="8">
-        <v>4</v>
-      </c>
-      <c r="M8">
-        <v>4</v>
+      <c r="M8" s="8">
+        <v>15</v>
       </c>
       <c r="N8" s="8">
         <v>20</v>
@@ -1836,28 +1847,28 @@
         <v>10</v>
       </c>
       <c r="F9" s="8">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G9" s="8">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H9" s="8">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="I9" s="8">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="J9" s="8">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="K9" s="8">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="L9" s="8">
-        <v>4</v>
-      </c>
-      <c r="M9">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="M9" s="8">
+        <v>18</v>
       </c>
       <c r="N9" s="8">
         <v>20</v>
@@ -1908,28 +1919,28 @@
         <v>10</v>
       </c>
       <c r="F10" s="8">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G10" s="8">
         <v>3</v>
       </c>
       <c r="H10" s="8">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="I10" s="8">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="J10" s="8">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="K10" s="8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L10" s="8">
-        <v>4</v>
-      </c>
-      <c r="M10">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="M10" s="8">
+        <v>15</v>
       </c>
       <c r="N10" s="8">
         <v>20</v>
@@ -1983,25 +1994,25 @@
         <v>6</v>
       </c>
       <c r="G11" s="8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H11" s="8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I11" s="8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J11" s="8">
         <v>2</v>
       </c>
       <c r="K11" s="8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L11" s="8">
-        <v>4</v>
-      </c>
-      <c r="M11">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="M11" s="8">
+        <v>16</v>
       </c>
       <c r="N11" s="8">
         <v>20</v>
@@ -2055,25 +2066,25 @@
         <v>6</v>
       </c>
       <c r="G12" s="8">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H12" s="8">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="I12" s="8">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="J12" s="8">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="K12" s="8">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="L12" s="8">
-        <v>4</v>
-      </c>
-      <c r="M12">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="M12" s="8">
+        <v>20</v>
       </c>
       <c r="N12" s="8">
         <v>20</v>
@@ -2127,7 +2138,7 @@
         <v>6</v>
       </c>
       <c r="G13" s="8">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H13" s="8">
         <v>3</v>
@@ -2136,16 +2147,16 @@
         <v>3</v>
       </c>
       <c r="J13" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K13" s="8">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L13" s="8">
-        <v>4</v>
-      </c>
-      <c r="M13">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="M13" s="8">
+        <v>9</v>
       </c>
       <c r="N13" s="8">
         <v>20</v>
@@ -2199,25 +2210,25 @@
         <v>6</v>
       </c>
       <c r="G14" s="8">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="H14" s="8">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="I14" s="8">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="J14" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="K14" s="8">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="L14" s="8">
-        <v>4</v>
-      </c>
-      <c r="M14">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="M14" s="8">
+        <v>20</v>
       </c>
       <c r="N14" s="8">
         <v>20</v>
@@ -2264,6 +2275,7 @@
       <c r="J15" s="9"/>
       <c r="K15" s="9"/>
       <c r="L15" s="9"/>
+      <c r="M15" s="9"/>
       <c r="N15" s="9"/>
       <c r="O15" s="9"/>
       <c r="P15" s="9"/>
@@ -2289,6 +2301,7 @@
       <c r="J16" s="9"/>
       <c r="K16" s="9"/>
       <c r="L16" s="9"/>
+      <c r="M16" s="9"/>
       <c r="N16" s="9"/>
       <c r="O16" s="9"/>
       <c r="P16" s="9"/>
@@ -2314,6 +2327,7 @@
       <c r="J17" s="9"/>
       <c r="K17" s="9"/>
       <c r="L17" s="9"/>
+      <c r="M17" s="9"/>
       <c r="N17" s="9"/>
       <c r="O17" s="9"/>
       <c r="P17" s="9"/>
@@ -2339,6 +2353,7 @@
       <c r="J18" s="9"/>
       <c r="K18" s="9"/>
       <c r="L18" s="9"/>
+      <c r="M18" s="9"/>
       <c r="N18" s="9"/>
       <c r="O18" s="9"/>
       <c r="P18" s="9"/>
@@ -2364,6 +2379,7 @@
       <c r="J19" s="9"/>
       <c r="K19" s="9"/>
       <c r="L19" s="9"/>
+      <c r="M19" s="9"/>
       <c r="N19" s="9"/>
       <c r="O19" s="9"/>
       <c r="P19" s="9"/>
@@ -2389,6 +2405,7 @@
       <c r="J20" s="9"/>
       <c r="K20" s="9"/>
       <c r="L20" s="9"/>
+      <c r="M20" s="9"/>
       <c r="N20" s="9"/>
       <c r="O20" s="9"/>
       <c r="P20" s="9"/>
@@ -2414,6 +2431,7 @@
       <c r="J21" s="9"/>
       <c r="K21" s="9"/>
       <c r="L21" s="9"/>
+      <c r="M21" s="9"/>
       <c r="N21" s="9"/>
       <c r="O21" s="9"/>
       <c r="P21" s="9"/>
@@ -2439,6 +2457,7 @@
       <c r="J22" s="9"/>
       <c r="K22" s="9"/>
       <c r="L22" s="9"/>
+      <c r="M22" s="9"/>
       <c r="N22" s="9"/>
       <c r="O22" s="9"/>
       <c r="P22" s="9"/>
@@ -2464,6 +2483,7 @@
       <c r="J23" s="9"/>
       <c r="K23" s="9"/>
       <c r="L23" s="9"/>
+      <c r="M23" s="9"/>
       <c r="N23" s="9"/>
       <c r="O23" s="9"/>
       <c r="P23" s="9"/>
@@ -2489,6 +2509,7 @@
       <c r="J24" s="9"/>
       <c r="K24" s="9"/>
       <c r="L24" s="9"/>
+      <c r="M24" s="9"/>
       <c r="N24" s="9"/>
       <c r="O24" s="9"/>
       <c r="P24" s="9"/>
@@ -2514,6 +2535,7 @@
       <c r="J25" s="9"/>
       <c r="K25" s="9"/>
       <c r="L25" s="9"/>
+      <c r="M25" s="9"/>
       <c r="N25" s="9"/>
       <c r="O25" s="9"/>
       <c r="P25" s="9"/>
@@ -2539,6 +2561,7 @@
       <c r="J26" s="9"/>
       <c r="K26" s="9"/>
       <c r="L26" s="9"/>
+      <c r="M26" s="9"/>
       <c r="N26" s="9"/>
       <c r="O26" s="9"/>
       <c r="P26" s="9"/>
@@ -2564,6 +2587,7 @@
       <c r="J27" s="9"/>
       <c r="K27" s="9"/>
       <c r="L27" s="9"/>
+      <c r="M27" s="9"/>
       <c r="N27" s="9"/>
       <c r="O27" s="9"/>
       <c r="P27" s="9"/>
@@ -2589,6 +2613,7 @@
       <c r="J28" s="9"/>
       <c r="K28" s="9"/>
       <c r="L28" s="9"/>
+      <c r="M28" s="9"/>
       <c r="N28" s="9"/>
       <c r="O28" s="9"/>
       <c r="P28" s="9"/>
@@ -2614,6 +2639,7 @@
       <c r="J29" s="9"/>
       <c r="K29" s="9"/>
       <c r="L29" s="9"/>
+      <c r="M29" s="9"/>
       <c r="N29" s="9"/>
       <c r="O29" s="9"/>
       <c r="P29" s="9"/>
@@ -2639,6 +2665,7 @@
       <c r="J30" s="9"/>
       <c r="K30" s="9"/>
       <c r="L30" s="9"/>
+      <c r="M30" s="9"/>
       <c r="N30" s="9"/>
       <c r="O30" s="9"/>
       <c r="P30" s="9"/>
@@ -2664,6 +2691,7 @@
       <c r="J31" s="9"/>
       <c r="K31" s="9"/>
       <c r="L31" s="9"/>
+      <c r="M31" s="9"/>
       <c r="N31" s="9"/>
       <c r="O31" s="9"/>
       <c r="P31" s="9"/>
@@ -2689,6 +2717,7 @@
       <c r="J32" s="9"/>
       <c r="K32" s="9"/>
       <c r="L32" s="9"/>
+      <c r="M32" s="9"/>
       <c r="N32" s="9"/>
       <c r="O32" s="9"/>
       <c r="P32" s="9"/>
@@ -2714,6 +2743,7 @@
       <c r="J33" s="9"/>
       <c r="K33" s="9"/>
       <c r="L33" s="9"/>
+      <c r="M33" s="9"/>
       <c r="N33" s="9"/>
       <c r="O33" s="9"/>
       <c r="P33" s="9"/>
@@ -2739,6 +2769,7 @@
       <c r="J34" s="9"/>
       <c r="K34" s="9"/>
       <c r="L34" s="9"/>
+      <c r="M34" s="9"/>
       <c r="N34" s="9"/>
       <c r="O34" s="9"/>
       <c r="P34" s="9"/>
@@ -2764,6 +2795,7 @@
       <c r="J35" s="9"/>
       <c r="K35" s="9"/>
       <c r="L35" s="9"/>
+      <c r="M35" s="9"/>
       <c r="N35" s="9"/>
       <c r="O35" s="9"/>
       <c r="P35" s="9"/>
@@ -2789,6 +2821,7 @@
       <c r="J36" s="9"/>
       <c r="K36" s="9"/>
       <c r="L36" s="9"/>
+      <c r="M36" s="9"/>
       <c r="N36" s="9"/>
       <c r="O36" s="9"/>
       <c r="P36" s="9"/>
@@ -2814,6 +2847,7 @@
       <c r="J37" s="9"/>
       <c r="K37" s="9"/>
       <c r="L37" s="9"/>
+      <c r="M37" s="9"/>
       <c r="N37" s="9"/>
       <c r="O37" s="9"/>
       <c r="P37" s="9"/>
@@ -2839,6 +2873,7 @@
       <c r="J38" s="9"/>
       <c r="K38" s="9"/>
       <c r="L38" s="9"/>
+      <c r="M38" s="9"/>
       <c r="N38" s="9"/>
       <c r="O38" s="9"/>
       <c r="P38" s="9"/>
@@ -2864,6 +2899,7 @@
       <c r="J39" s="9"/>
       <c r="K39" s="9"/>
       <c r="L39" s="9"/>
+      <c r="M39" s="9"/>
       <c r="N39" s="9"/>
       <c r="O39" s="9"/>
       <c r="P39" s="9"/>
@@ -2889,6 +2925,7 @@
       <c r="J40" s="9"/>
       <c r="K40" s="9"/>
       <c r="L40" s="9"/>
+      <c r="M40" s="9"/>
       <c r="N40" s="9"/>
       <c r="O40" s="9"/>
       <c r="P40" s="9"/>
@@ -2914,6 +2951,7 @@
       <c r="J41" s="9"/>
       <c r="K41" s="9"/>
       <c r="L41" s="9"/>
+      <c r="M41" s="9"/>
       <c r="N41" s="9"/>
       <c r="O41" s="9"/>
       <c r="P41" s="9"/>

</xml_diff>